<commit_message>
Improve What3Words form guidance
</commit_message>
<xml_diff>
--- a/forms/wwm_kobo_current.xlsx
+++ b/forms/wwm_kobo_current.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Optional. Enter the three words for this sampling site, for example filled.count.soap or ///filled.count.soap.</t>
+          <t>Optional. For an Atacama Desert sampling site, select the exact 3 m square in the what3words app or map and paste it here, e.g. ///word.word.word.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>filled.count.soap</t>
+          <t>///word.word.word</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">

</xml_diff>